<commit_message>
Paquetes de arranque por docente y cronograma del 15 de octubre
Carpetas docentes/comercial y docentes/administrativo con el brief del
docente, cronograma, sesiones de Teams por perfil, temario, guías, kit,
manual de puntajes, ajustes, política y plantillas. Fechas del Taller 1
y 2 comercial actualizadas en los documentos de ajustes y de propuesta.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja1vbRoiAwxTq3mLFGrVau
</commit_message>
<xml_diff>
--- a/plan-y-cronograma/Citaciones de Teams · textos.xlsx
+++ b/plan-y-cronograma/Citaciones de Teams · textos.xlsx
@@ -71,28 +71,50 @@
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
+    <t xml:space="preserve">Administrativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encuentro 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miércoles 21 de octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8:00 a.m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9:30 a.m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 h 30 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no consulta tus sistemas (todavía)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrancamos desde cero. Qué es la inteligencia artificial, cómo funciona por dentro y por qué cita normas que no existen. Vas a abrir la herramienta por primera vez, acompañado, y a convertir las notas de un comité en un acta con decisiones, responsables y fechas. Trae una tarea tuya que te quite tiempo.
+Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comercial</t>
   </si>
   <si>
-    <t xml:space="preserve">T1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encuentro 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viernes 16 de octubre</t>
+    <t xml:space="preserve">23/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">viernes 23 de octubre</t>
   </si>
   <si>
     <t xml:space="preserve">7:30 a.m.</t>
   </si>
   <si>
     <t xml:space="preserve">9:00 a.m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 h 30 min</t>
   </si>
   <si>
     <t xml:space="preserve">Super Humanos · Taller 1 · La IA no sabe nada de tu cliente (todavía)</t>
@@ -102,28 +124,6 @@
 Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
   </si>
   <si>
-    <t xml:space="preserve">Administrativo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">miércoles 21 de octubre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8:00 a.m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9:30 a.m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no consulta tus sistemas (todavía)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrancamos desde cero. Qué es la inteligencia artificial, cómo funciona por dentro y por qué cita normas que no existen. Vas a abrir la herramienta por primera vez, acompañado, y a convertir las notas de un comité en un acta con decisiones, responsables y fechas. Trae una tarea tuya que te quite tiempo.
-Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Consultorio</t>
   </si>
   <si>
@@ -145,35 +145,48 @@
     <t xml:space="preserve">Encuentro 2</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viernes 23 de octubre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no sabe nada de tu cliente (todavía) (parte 2)</t>
+    <t xml:space="preserve">28/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miércoles 28 de octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no consulta tus sistemas (todavía) (parte 2)</t>
   </si>
   <si>
     <t xml:space="preserve">Hoy trabajas tu propia tarea. Traes la que elegiste en el encuentro anterior, la mides, la mejoras y la vuelves a medir. Tres o cuatro personas comparten su pantalla y el grupo retroalimenta.
 Al final abrimos la evaluación del taller: diez preguntas, cinco minutos, suma 30 puntos.</t>
   </si>
   <si>
-    <t xml:space="preserve">28/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">miércoles 28 de octubre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no consulta tus sistemas (todavía) (parte 2)</t>
+    <t xml:space="preserve">30/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">viernes 30 de octubre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Humanos · Taller 1 · La IA no sabe nada de tu cliente (todavía) (parte 2)</t>
   </si>
   <si>
     <t xml:space="preserve">T2</t>
   </si>
   <si>
-    <t xml:space="preserve">06/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viernes 6 de noviembre</t>
+    <t xml:space="preserve">11/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miércoles 11 de noviembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Humanos · Taller 2 · Tres días armando el reporte, cero analizándolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si el mes se te va consolidando archivos, este taller es para ti. Vas a juntar tres archivos con formatos distintos, verificar que los totales cuadren y salir con el informe de una página listo para el comité.
+Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">viernes 13 de noviembre</t>
   </si>
   <si>
     <t xml:space="preserve">Super Humanos · Taller 2 · Tu cartera tiene cosas que contarte</t>
@@ -183,44 +196,31 @@
 Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
   </si>
   <si>
-    <t xml:space="preserve">11/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">miércoles 11 de noviembre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Humanos · Taller 2 · Tres días armando el reporte, cero analizándolo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si el mes se te va consolidando archivos, este taller es para ti. Vas a juntar tres archivos con formatos distintos, verificar que los totales cuadren y salir con el informe de una página listo para el comité.
-Encuentro 1 de 2. Hora y media, con la herramienta abierta. La grabación queda en la plataforma al día siguiente.</t>
+    <t xml:space="preserve">17/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">martes 17 de noviembre</t>
   </si>
   <si>
     <t xml:space="preserve">Super Humanos · Consultorio del Taller 2</t>
   </si>
   <si>
-    <t xml:space="preserve">13/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viernes 13 de noviembre</t>
+    <t xml:space="preserve">18/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miércoles 18 de noviembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Super Humanos · Taller 2 · Tres días armando el reporte, cero analizándolo (parte 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">viernes 20 de noviembre</t>
   </si>
   <si>
     <t xml:space="preserve">Super Humanos · Taller 2 · Tu cartera tiene cosas que contarte (parte 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">martes 17 de noviembre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">miércoles 18 de noviembre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Super Humanos · Taller 2 · Tres días armando el reporte, cero analizándolo (parte 2)</t>
   </si>
   <si>
     <t xml:space="preserve">T3</t>
@@ -1486,10 +1486,10 @@
         <v>32</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>33</v>
@@ -1501,7 +1501,7 @@
         <v>35</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>37</v>
@@ -1524,10 +1524,10 @@
         <v>38</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H14" s="12" t="s">
         <v>20</v>
@@ -1539,7 +1539,7 @@
         <v>22</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L14" s="14" t="s">
         <v>42</v>
@@ -1562,10 +1562,10 @@
         <v>32</v>
       </c>
       <c r="F15" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>59</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>60</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>33</v>
@@ -1577,7 +1577,7 @@
         <v>35</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>37</v>
@@ -1629,7 +1629,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>64</v>
@@ -1644,10 +1644,10 @@
         <v>66</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J17" s="8" t="s">
         <v>22</v>
@@ -1667,7 +1667,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>64</v>
@@ -1705,7 +1705,7 @@
         <v>14</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>64</v>
@@ -1720,10 +1720,10 @@
         <v>73</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J19" s="8" t="s">
         <v>22</v>
@@ -1743,7 +1743,7 @@
         <v>14</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>64</v>
@@ -1758,10 +1758,10 @@
         <v>77</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J20" s="12" t="s">
         <v>22</v>
@@ -1781,7 +1781,7 @@
         <v>14</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>64</v>
@@ -1819,7 +1819,7 @@
         <v>14</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>64</v>
@@ -1834,10 +1834,10 @@
         <v>82</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>22</v>
@@ -1857,7 +1857,7 @@
         <v>14</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>84</v>
@@ -1872,10 +1872,10 @@
         <v>86</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J23" s="8" t="s">
         <v>22</v>
@@ -1895,7 +1895,7 @@
         <v>14</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>84</v>
@@ -1910,10 +1910,10 @@
         <v>90</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J24" s="12" t="s">
         <v>22</v>
@@ -1933,7 +1933,7 @@
         <v>14</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>84</v>
@@ -1971,7 +1971,7 @@
         <v>14</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>84</v>
@@ -2009,7 +2009,7 @@
         <v>14</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>84</v>
@@ -2024,10 +2024,10 @@
         <v>99</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J27" s="8" t="s">
         <v>22</v>
@@ -2047,7 +2047,7 @@
         <v>14</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>84</v>
@@ -2062,10 +2062,10 @@
         <v>102</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J28" s="12" t="s">
         <v>22</v>
@@ -2085,7 +2085,7 @@
         <v>14</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>104</v>
@@ -2100,10 +2100,10 @@
         <v>106</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J29" s="8" t="s">
         <v>22</v>
@@ -2123,7 +2123,7 @@
         <v>14</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>104</v>
@@ -2138,10 +2138,10 @@
         <v>110</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I30" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J30" s="12" t="s">
         <v>22</v>
@@ -2161,7 +2161,7 @@
         <v>14</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>104</v>
@@ -2199,7 +2199,7 @@
         <v>14</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>104</v>
@@ -2214,10 +2214,10 @@
         <v>115</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J32" s="12" t="s">
         <v>22</v>
@@ -2237,7 +2237,7 @@
         <v>14</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>104</v>
@@ -2275,7 +2275,7 @@
         <v>14</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>104</v>
@@ -2290,10 +2290,10 @@
         <v>120</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J34" s="12" t="s">
         <v>22</v>
@@ -2313,7 +2313,7 @@
         <v>14</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>122</v>
@@ -2328,10 +2328,10 @@
         <v>124</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J35" s="8" t="s">
         <v>22</v>
@@ -2351,7 +2351,7 @@
         <v>14</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>122</v>
@@ -2366,10 +2366,10 @@
         <v>128</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>22</v>
@@ -2389,7 +2389,7 @@
         <v>14</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>122</v>
@@ -2427,7 +2427,7 @@
         <v>14</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>122</v>
@@ -2442,10 +2442,10 @@
         <v>131</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>22</v>
@@ -2465,7 +2465,7 @@
         <v>14</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>122</v>
@@ -2503,7 +2503,7 @@
         <v>14</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>122</v>
@@ -2518,10 +2518,10 @@
         <v>136</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>22</v>
@@ -2626,7 +2626,7 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>149</v>
@@ -2634,7 +2634,7 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>150</v>

</xml_diff>